<commit_message>
Changed update Amrfinder database (august 2026)
</commit_message>
<xml_diff>
--- a/Illumina_only_pipe/src/singularity/MAJ_tools_2026.xlsx
+++ b/Illumina_only_pipe/src/singularity/MAJ_tools_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afischer\Documents\Projets\2.Coding_projects\42.MAJ_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D35395F-A925-48D0-AFA3-022E1FE872AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B463AE-69B3-4F8F-9D23-B10B687E5C9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6FC7DDD9-4E5A-4BF4-8DFF-E17A0FA680F0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6FC7DDD9-4E5A-4BF4-8DFF-E17A0FA680F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Tools" sheetId="1" r:id="rId1"/>
@@ -421,9 +421,6 @@
     <t>Replace Circlator by dnaapler [interesting for Nanopore contigs]</t>
   </si>
   <si>
-    <t>2026-05-15.1</t>
-  </si>
-  <si>
     <r>
       <t>The </t>
     </r>
@@ -873,6 +870,9 @@
   </si>
   <si>
     <t>Note : Please after update or any creation of the container, check that plasmid results are output by the tool (plasmid_AA002.fasta;…) If not, then command to initiate mob-suite db has failed.</t>
+  </si>
+  <si>
+    <t>2026-08-07.1</t>
   </si>
 </sst>
 </file>
@@ -1939,7 +1939,7 @@
         <v>98</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -2171,7 +2171,7 @@
         <v>115</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -2191,16 +2191,16 @@
         <v>18</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F3" s="20" t="s">
         <v>116</v>
@@ -2215,25 +2215,25 @@
         <v>20</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C4" s="25" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F4" s="27" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G4" s="25" t="s">
         <v>69</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -2247,19 +2247,19 @@
         <v>69</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E5" s="30">
         <v>45778</v>
       </c>
       <c r="F5" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="G5" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="H5" s="25" t="s">
         <v>142</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="H5" s="25" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -2273,10 +2273,10 @@
         <v>69</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="E6" s="28">
-        <v>46157</v>
+        <v>46241</v>
       </c>
       <c r="F6" s="25" t="s">
         <v>119</v>
@@ -2327,13 +2327,13 @@
         <v>45268</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G8" s="25" t="s">
         <v>69</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -2353,25 +2353,25 @@
         <v>30</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C10" s="25" t="s">
         <v>69</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E10" s="28">
         <v>46171</v>
       </c>
       <c r="F10" s="25" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G10" s="25" t="s">
         <v>69</v>
       </c>
       <c r="H10" s="25" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -2406,42 +2406,42 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B13" s="35" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B14" s="35" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B15" s="35" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B18" s="35" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B22" s="36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>